<commit_message>
Add SSRR proceedings to RoboPaper Atlas
</commit_message>
<xml_diff>
--- a/by_venue/RA-P.xlsx
+++ b/by_venue/RA-P.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="211">
   <si>
     <t>venue</t>
   </si>
@@ -103,19 +103,19 @@
     <t>NanoCockpit: Performance-optimized Application Framework for AI-based Autonomous Nanorobotics</t>
   </si>
   <si>
-    <t>Out-of-Distribution Image Detection With Classified Generative Adversarial Network (C-GAN) in an Industrial System</t>
+    <t>Out-of-Distribution Image Detection With Classified Generative Adversarial Network in an Industrial System</t>
   </si>
   <si>
     <t>Physical Simulation of Marsupial UAV-UGV Systems Connected by a Variable-Length Hanging Tether</t>
   </si>
   <si>
-    <t>RSLCPP - Deterministic Simulations Using ROS 2</t>
+    <t>RSLCPP—Deterministic Simulations Using ROS 2</t>
   </si>
   <si>
     <t>Reducing Heavy Physical Labor With Robotics: Aviation Industry Case Study of Aircraft Engine Fan Blade Repair With Blending</t>
   </si>
   <si>
-    <t>Reproducibility of Legacy ROS-based Research Code through Transparent Docker Integration</t>
+    <t>Reproducibility of Legacy ROS-Based Research Code Through Transparent Docker Integration</t>
   </si>
   <si>
     <t>Soft Finger AI Enabled Hand (SofIA): Design and Applications of an Open Source Soft Gripper</t>
@@ -124,7 +124,7 @@
     <t>Toward Reliable Bin-Picking: Collision-Aware Robotic Design and Control Strategy for Heavily Cluttered Environment</t>
   </si>
   <si>
-    <t>You Only Orient Once (YOOO): Vision-Driven Robotic Cable Insertion for Automotive Wiring Harness Assembly</t>
+    <t>You Only Orient Once: Vision-Driven Robotic Cable Insertion for Automotive Wiring Harness Assembly</t>
   </si>
   <si>
     <t>iChores: Intuitive Collaboration With Household Robots in Everyday Settings</t>
@@ -208,7 +208,7 @@
     <t>Seunghwan Um; Yeong Gwang Son; Jaeyoon Shim; Hyouk Ryeol Choi</t>
   </si>
   <si>
-    <t>Abdelrahman Mahmoud; Rodolfo Verde; Volker Willert; Tobias Kaupp</t>
+    <t>Abdelrahman Mahmoud; Rodolfo Verde; Tobias Kaupp; Volker Willert</t>
   </si>
   <si>
     <t>Antonio Galiza Cerdeira Gonzalez; Peter A. Hoenig; Matthias Hirschmanner; Karolina Zrobek; Pawel Gajewski; Tessa Pulli; Petr Vanc; Simon Dratva; Gabriela Šejnová; Radoslav Škoviera; Karla Stepanova; Michal Vavrečka; Markus Vincze; Bipin Indurkhya</t>
@@ -517,30 +517,36 @@
     <t>https://doi.org/10.1109/rap.2025.3632798</t>
   </si>
   <si>
+    <t>86-91</t>
+  </si>
+  <si>
+    <t>29-34</t>
+  </si>
+  <si>
+    <t>23-28</t>
+  </si>
+  <si>
+    <t>103-107</t>
+  </si>
+  <si>
     <t>1-6</t>
   </si>
   <si>
-    <t>29-34</t>
-  </si>
-  <si>
-    <t>23-28</t>
-  </si>
-  <si>
-    <t>103-107</t>
-  </si>
-  <si>
     <t>40-44</t>
   </si>
   <si>
+    <t>81-85</t>
+  </si>
+  <si>
+    <t>45-49</t>
+  </si>
+  <si>
+    <t>71-75</t>
+  </si>
+  <si>
     <t>1-5</t>
   </si>
   <si>
-    <t>45-49</t>
-  </si>
-  <si>
-    <t>71-75</t>
-  </si>
-  <si>
     <t>108-112</t>
   </si>
   <si>
@@ -553,10 +559,25 @@
     <t>50-54</t>
   </si>
   <si>
+    <t>97-102</t>
+  </si>
+  <si>
+    <t>113-117</t>
+  </si>
+  <si>
+    <t>118-122</t>
+  </si>
+  <si>
     <t>123-127</t>
   </si>
   <si>
+    <t>92-96</t>
+  </si>
+  <si>
     <t>35-39</t>
+  </si>
+  <si>
+    <t>76-80</t>
   </si>
   <si>
     <t>60-65</t>
@@ -1046,7 +1067,7 @@
         <v>167</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="M2" t="s">
         <v>13</v>
@@ -1084,7 +1105,7 @@
         <v>168</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="M3" t="s">
         <v>13</v>
@@ -1122,7 +1143,7 @@
         <v>169</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="M4" t="s">
         <v>13</v>
@@ -1183,7 +1204,7 @@
         <v>143</v>
       </c>
       <c r="J6" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="M6" t="s">
         <v>13</v>
@@ -1218,10 +1239,10 @@
         <v>144</v>
       </c>
       <c r="J7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="M7" t="s">
         <v>13</v>
@@ -1256,10 +1277,10 @@
         <v>145</v>
       </c>
       <c r="J8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="M8" t="s">
         <v>13</v>
@@ -1291,10 +1312,10 @@
         <v>146</v>
       </c>
       <c r="J9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M9" t="s">
         <v>13</v>
@@ -1329,10 +1350,10 @@
         <v>147</v>
       </c>
       <c r="J10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="M10" t="s">
         <v>13</v>
@@ -1361,7 +1382,7 @@
         <v>148</v>
       </c>
       <c r="J11" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="M11" t="s">
         <v>13</v>
@@ -1396,7 +1417,7 @@
         <v>149</v>
       </c>
       <c r="J12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="M12" t="s">
         <v>13</v>
@@ -1431,10 +1452,10 @@
         <v>150</v>
       </c>
       <c r="J13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="M13" t="s">
         <v>13</v>
@@ -1469,10 +1490,10 @@
         <v>151</v>
       </c>
       <c r="J14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="M14" t="s">
         <v>13</v>
@@ -1507,10 +1528,10 @@
         <v>152</v>
       </c>
       <c r="J15" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="M15" t="s">
         <v>13</v>
@@ -1542,10 +1563,10 @@
         <v>153</v>
       </c>
       <c r="J16" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="M16" t="s">
         <v>13</v>
@@ -1574,7 +1595,7 @@
         <v>154</v>
       </c>
       <c r="J17" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="M17" t="s">
         <v>13</v>
@@ -1609,7 +1630,7 @@
         <v>155</v>
       </c>
       <c r="J18" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="M18" t="s">
         <v>13</v>
@@ -1635,7 +1656,7 @@
         <v>156</v>
       </c>
       <c r="J19" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="M19" t="s">
         <v>13</v>
@@ -1667,7 +1688,7 @@
         <v>157</v>
       </c>
       <c r="J20" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="M20" t="s">
         <v>13</v>
@@ -1702,10 +1723,10 @@
         <v>158</v>
       </c>
       <c r="J21" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="M21" t="s">
         <v>13</v>
@@ -1734,7 +1755,7 @@
         <v>159</v>
       </c>
       <c r="J22" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="M22" t="s">
         <v>13</v>
@@ -1769,10 +1790,10 @@
         <v>160</v>
       </c>
       <c r="J23" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="M23" t="s">
         <v>13</v>
@@ -1807,10 +1828,10 @@
         <v>161</v>
       </c>
       <c r="J24" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="M24" t="s">
         <v>13</v>
@@ -1845,10 +1866,10 @@
         <v>162</v>
       </c>
       <c r="J25" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="M25" t="s">
         <v>13</v>
@@ -1883,10 +1904,10 @@
         <v>163</v>
       </c>
       <c r="J26" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="M26" t="s">
         <v>13</v>
@@ -1921,10 +1942,10 @@
         <v>164</v>
       </c>
       <c r="J27" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="M27" t="s">
         <v>13</v>
@@ -1959,10 +1980,10 @@
         <v>165</v>
       </c>
       <c r="J28" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="M28" t="s">
         <v>13</v>
@@ -1997,10 +2018,10 @@
         <v>166</v>
       </c>
       <c r="J29" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="M29" t="s">
         <v>13</v>

</xml_diff>